<commit_message>
add SPI library, ready to use, example using SRAM and changes of GPIO output
</commit_message>
<xml_diff>
--- a/documentation/pines y puertos disponibles.xlsx
+++ b/documentation/pines y puertos disponibles.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\OneDrive\Escritorio\STMCube_Courses\Bare-Metal\Proyecto_personal\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\sebas\Desktop\STMCube_Courses\Bare-Metal\Proyecto_personal\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91416C6-66BA-461E-AB09-50CA7C208BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23148" windowHeight="9360"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -19,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="171">
   <si>
     <t>Port C</t>
   </si>
@@ -518,12 +510,42 @@
   </si>
   <si>
     <t>UART2 RX (only for uart)</t>
+  </si>
+  <si>
+    <t>SPI</t>
+  </si>
+  <si>
+    <t>SPI1_SCK</t>
+  </si>
+  <si>
+    <t>SPI1_MISO</t>
+  </si>
+  <si>
+    <t>SPI1_MOSI</t>
+  </si>
+  <si>
+    <t>SPI2_SCK</t>
+  </si>
+  <si>
+    <t>SPI2_MISO</t>
+  </si>
+  <si>
+    <t>SPI2_MOSI</t>
+  </si>
+  <si>
+    <t>SPI5_MISO</t>
+  </si>
+  <si>
+    <t>SPI5_MOSI</t>
+  </si>
+  <si>
+    <t>SPI5_SCK</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -557,7 +579,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -690,8 +712,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -808,17 +836,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -868,56 +885,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -927,7 +899,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -965,42 +936,22 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1018,12 +969,6 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1032,41 +977,16 @@
     <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1075,6 +995,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1094,19 +1019,13 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1121,7 +1040,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1136,15 +1055,13 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1153,9 +1070,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFA162D0"/>
       <color rgb="FFFF4343"/>
       <color rgb="FFFF6600"/>
-      <color rgb="FFA162D0"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1183,7 +1100,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="CuadroTexto 1"/>
+            <xdr:cNvPr id="2" name="CuadroTexto 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -1485,7 +1408,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="3" name="CuadroTexto 2"/>
+            <xdr:cNvPr id="3" name="CuadroTexto 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -1750,7 +1679,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="CuadroTexto 3"/>
+            <xdr:cNvPr id="4" name="CuadroTexto 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -1946,7 +1881,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="5" name="CuadroTexto 4"/>
+            <xdr:cNvPr id="5" name="CuadroTexto 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -2166,13 +2107,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>35</xdr:col>
-      <xdr:colOff>749505</xdr:colOff>
+      <xdr:colOff>745695</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>82280</xdr:rowOff>
+      <xdr:rowOff>95615</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Imagen 5"/>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -2207,7 +2154,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="7" name="CuadroTexto 6"/>
+            <xdr:cNvPr id="7" name="CuadroTexto 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -2564,7 +2517,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="8" name="CuadroTexto 7"/>
+            <xdr:cNvPr id="8" name="CuadroTexto 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -2773,7 +2732,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="9" name="CuadroTexto 8"/>
+            <xdr:cNvPr id="9" name="CuadroTexto 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -3144,7 +3109,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="10" name="CuadroTexto 9"/>
+            <xdr:cNvPr id="10" name="CuadroTexto 9">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -3508,7 +3479,13 @@
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="11" name="CuadroTexto 10"/>
+            <xdr:cNvPr id="11" name="CuadroTexto 10">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
             <xdr:cNvSpPr txBox="1"/>
           </xdr:nvSpPr>
           <xdr:spPr>
@@ -3863,7 +3840,13 @@
     <xdr:ext cx="2740494" cy="352597"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="CuadroTexto 11"/>
+        <xdr:cNvPr id="12" name="CuadroTexto 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -3932,7 +3915,13 @@
     <xdr:ext cx="2572499" cy="352597"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="CuadroTexto 13"/>
+        <xdr:cNvPr id="14" name="CuadroTexto 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -4000,13 +3989,19 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>29</xdr:col>
-      <xdr:colOff>583175</xdr:colOff>
+      <xdr:colOff>586985</xdr:colOff>
       <xdr:row>65</xdr:row>
-      <xdr:rowOff>4702</xdr:rowOff>
+      <xdr:rowOff>16133</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Imagen 14" descr="C:\Users\sebas\AppData\Local\Packages\Microsoft.Windows.Photos_8wekyb3d8bbwe\TempState\ShareServiceTempFolder\pin-out nucleoF411RE.jpeg"/>
+        <xdr:cNvPr id="15" name="Imagen 14" descr="C:\Users\sebas\AppData\Local\Packages\Microsoft.Windows.Photos_8wekyb3d8bbwe\TempState\ShareServiceTempFolder\pin-out nucleoF411RE.jpeg">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -4028,6 +4023,67 @@
         <a:xfrm>
           <a:off x="16315616" y="7307470"/>
           <a:ext cx="5936934" cy="4834803"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>737420</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>49160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>741230</xdr:colOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>21876</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Imagen 12" descr="Understanding SPI Clock Signals: Polarity, Phase, Clock Edges, and SPI  Modes - Total Phase">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E8538161-4916-2414-C1B0-C43B7885036B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="20377355" y="15436644"/>
+          <a:ext cx="4727104" cy="2905433"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4345,8 +4401,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U78"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Y87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -4360,401 +4416,371 @@
     <col min="17" max="18" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="76" t="s">
+    <row r="1" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B1" s="57" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-    </row>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B2" s="63" t="s">
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="63" t="s">
+      <c r="C2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="63" t="s">
+      <c r="E2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-    </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B3" s="9">
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B3" s="8">
         <v>0</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>2</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="49"/>
-      <c r="R3" s="49"/>
-      <c r="S3" s="49"/>
-      <c r="T3" s="49"/>
-    </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B4" s="9">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B4" s="8">
         <v>1</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>1</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>1</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="P4" s="49"/>
-      <c r="Q4" s="49"/>
-      <c r="R4" s="49"/>
-      <c r="S4" s="49"/>
-      <c r="T4" s="49"/>
-    </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B5" s="9">
+      <c r="E4" s="8"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+    </row>
+    <row r="5" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B5" s="8">
         <v>4</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="8">
         <v>2</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>2</v>
       </c>
-      <c r="E5" s="9"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="P5" s="49"/>
-      <c r="Q5" s="49"/>
-      <c r="R5" s="49"/>
-      <c r="S5" s="49"/>
-      <c r="T5" s="49"/>
-    </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B6" s="9">
+      <c r="E5" s="8"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+    </row>
+    <row r="6" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B6" s="8">
         <v>5</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="8">
         <v>4</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>3</v>
       </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="P6" s="49"/>
-      <c r="Q6" s="49"/>
-      <c r="R6" s="49"/>
-      <c r="S6" s="49"/>
-      <c r="T6" s="49"/>
-    </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B7" s="9">
+      <c r="E6" s="8"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+    </row>
+    <row r="7" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B7" s="8">
         <v>6</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>5</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>4</v>
       </c>
-      <c r="E7" s="9"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
-    </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B8" s="9">
+      <c r="E7" s="8"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+    </row>
+    <row r="8" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B8" s="8">
         <v>7</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="8">
         <v>6</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>5</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-    </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B9" s="9">
+      <c r="E8" s="8"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+    </row>
+    <row r="9" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B9" s="8">
         <v>8</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="8">
         <v>7</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <v>6</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-    </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B10" s="9">
+      <c r="E9" s="8"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B10" s="8">
         <v>9</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>8</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <v>7</v>
       </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-    </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B11" s="9">
+      <c r="E10" s="8"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B11" s="8">
         <v>10</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="8">
         <v>9</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <v>8</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B12" s="9">
+      <c r="E11" s="8"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B12" s="8">
         <v>11</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>10</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <v>9</v>
       </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-    </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B13" s="9">
+      <c r="E12" s="8"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B13" s="8">
         <v>12</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>12</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>10</v>
       </c>
-      <c r="E13" s="9"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="O13" s="69" t="s">
+      <c r="E13" s="8"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="O13" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="P13" s="69"/>
-      <c r="Q13" s="69"/>
-      <c r="R13" s="69"/>
-      <c r="S13" s="69"/>
-    </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B14" s="9">
+      <c r="P13" s="50"/>
+      <c r="Q13" s="50"/>
+      <c r="R13" s="50"/>
+      <c r="S13" s="50"/>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B14" s="8">
         <v>15</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>13</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="6">
         <v>11</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="O14" s="58" t="s">
+      <c r="E14" s="8"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="O14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="P14" s="58" t="s">
+      <c r="P14" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Q14" s="58" t="s">
+      <c r="Q14" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="R14" s="68" t="s">
+      <c r="R14" s="49" t="s">
         <v>136</v>
       </c>
-      <c r="S14" s="68"/>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B15" s="9"/>
-      <c r="C15" s="9">
+      <c r="S14" s="49"/>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8">
         <v>14</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <v>12</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="O15" s="58" t="s">
+      <c r="E15" s="8"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="O15" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="P15" s="58">
+      <c r="P15" s="4">
         <v>16</v>
       </c>
-      <c r="Q15" s="58" t="s">
+      <c r="Q15" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R15" s="74" t="s">
+      <c r="R15" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="S15" s="75"/>
-    </row>
-    <row r="16" spans="2:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="10"/>
-      <c r="C16" s="10">
+      <c r="S15" s="56"/>
+    </row>
+    <row r="16" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9">
         <v>15</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="7">
         <v>13</v>
       </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="O16" s="58" t="s">
+      <c r="E16" s="9"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="O16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="P16" s="58">
+      <c r="P16" s="4">
         <v>32</v>
       </c>
-      <c r="Q16" s="58" t="s">
+      <c r="Q16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R16" s="74" t="s">
+      <c r="R16" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="S16" s="75"/>
+      <c r="S16" s="56"/>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B17" s="6"/>
-      <c r="O17" s="58" t="s">
+      <c r="B17" s="5"/>
+      <c r="O17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P17" s="58">
+      <c r="P17" s="4">
         <v>16</v>
       </c>
-      <c r="Q17" s="58" t="s">
+      <c r="Q17" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R17" s="74" t="s">
+      <c r="R17" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="S17" s="75"/>
+      <c r="S17" s="56"/>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="O18" s="58" t="s">
+      <c r="O18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P18" s="58">
+      <c r="P18" s="4">
         <v>16</v>
       </c>
-      <c r="Q18" s="58" t="s">
+      <c r="Q18" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R18" s="74" t="s">
+      <c r="R18" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="S18" s="75"/>
+      <c r="S18" s="56"/>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="O19" s="58" t="s">
+      <c r="O19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="P19" s="58">
+      <c r="P19" s="4">
         <v>16</v>
       </c>
-      <c r="Q19" s="58" t="s">
+      <c r="Q19" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="R19" s="74" t="s">
+      <c r="R19" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="S19" s="75"/>
+      <c r="S19" s="56"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B20" s="57" t="s">
+      <c r="B20" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D20" s="88" t="s">
+      <c r="D20" s="57" t="s">
         <v>153</v>
       </c>
-      <c r="E20" s="88"/>
-      <c r="F20" s="28" t="s">
+      <c r="E20" s="57"/>
+      <c r="F20" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G20" s="43" t="s">
+      <c r="G20" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="H20" s="54" t="s">
+      <c r="H20" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="I20" s="54" t="s">
+      <c r="I20" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
-      <c r="M20" s="49"/>
-      <c r="N20" s="49"/>
+      <c r="J20" s="3" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
@@ -4763,23 +4789,19 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="36" t="s">
+      <c r="F21" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="G21" s="65" t="s">
+      <c r="G21" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="37" t="s">
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="O21" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="P21" s="37" t="s">
+      <c r="P21" s="28" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4790,65 +4812,57 @@
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="36" t="s">
+      <c r="F22" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="G22" s="65" t="s">
+      <c r="G22" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="26"/>
-      <c r="I22" s="26"/>
-      <c r="J22" s="49"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="49"/>
-      <c r="M22" s="49"/>
-      <c r="N22" s="49"/>
-      <c r="O22" s="30" t="s">
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="O22" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="P22" s="35" t="s">
+      <c r="P22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="R22" s="70" t="s">
+      <c r="R22" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="S22" s="70"/>
-      <c r="T22" s="70"/>
+      <c r="S22" s="51"/>
+      <c r="T22" s="51"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>158</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <v>2</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="55" t="s">
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="I23" s="26"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="52"/>
-      <c r="N23" s="52"/>
-      <c r="O23" s="30" t="s">
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="O23" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="P23" s="30" t="s">
+      <c r="P23" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="R23" s="48" t="s">
+      <c r="R23" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="S23" s="48" t="s">
+      <c r="S23" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="T23" s="48" t="s">
+      <c r="T23" s="4" t="s">
         <v>132</v>
       </c>
     </row>
@@ -4856,36 +4870,32 @@
       <c r="A24" t="s">
         <v>158</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="10">
         <v>3</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="56" t="s">
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="I24" s="62"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="49"/>
-      <c r="M24" s="49"/>
-      <c r="N24" s="49"/>
-      <c r="O24" s="13" t="s">
+      <c r="I24" s="40"/>
+      <c r="J24" s="1"/>
+      <c r="O24" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="P24" s="13" t="s">
+      <c r="P24" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="R24" s="66" t="s">
+      <c r="R24" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="S24" s="67" t="s">
+      <c r="S24" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="T24" s="67" t="s">
+      <c r="T24" s="45" t="s">
         <v>133</v>
       </c>
       <c r="U24" t="s">
@@ -4896,41 +4906,37 @@
       <c r="B25" s="3">
         <v>4</v>
       </c>
-      <c r="C25" s="81" t="s">
+      <c r="C25" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="83" t="s">
+      <c r="D25" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="E25" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F25" s="36" t="s">
+      <c r="F25" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="26"/>
-      <c r="H25" s="59" t="s">
+      <c r="G25" s="1"/>
+      <c r="H25" s="38" t="s">
         <v>145</v>
       </c>
-      <c r="I25" s="26"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="49"/>
-      <c r="M25" s="49"/>
-      <c r="N25" s="49"/>
-      <c r="O25" s="13" t="s">
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="O25" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="P25" s="13" t="s">
+      <c r="P25" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="R25" s="66" t="s">
+      <c r="R25" s="44" t="s">
         <v>91</v>
       </c>
-      <c r="S25" s="67" t="s">
+      <c r="S25" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="T25" s="67" t="s">
+      <c r="T25" s="45" t="s">
         <v>133</v>
       </c>
       <c r="U25" t="s">
@@ -4938,41 +4944,39 @@
       </c>
     </row>
     <row r="26" spans="1:21" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="33">
+      <c r="B26" s="26">
         <v>5</v>
       </c>
-      <c r="C26" s="81"/>
-      <c r="D26" s="83"/>
-      <c r="E26" s="23" t="s">
+      <c r="C26" s="60"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="36" t="s">
+      <c r="F26" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="49"/>
-      <c r="O26" s="30" t="s">
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="O26" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="P26" s="30" t="s">
+      <c r="P26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="R26" s="38" t="s">
+      <c r="R26" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="S26" s="39" t="s">
+      <c r="S26" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="T26" s="39" t="s">
+      <c r="T26" s="30" t="s">
         <v>134</v>
       </c>
     </row>
@@ -4980,35 +4984,33 @@
       <c r="B27" s="3">
         <v>6</v>
       </c>
-      <c r="C27" s="81"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="23" t="s">
+      <c r="C27" s="60"/>
+      <c r="D27" s="62"/>
+      <c r="E27" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="F27" s="36" t="s">
+      <c r="F27" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
-      <c r="M27" s="49"/>
-      <c r="N27" s="49"/>
-      <c r="O27" s="30" t="s">
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="O27" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="P27" s="30" t="s">
+      <c r="P27" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="R27" s="38" t="s">
+      <c r="R27" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="S27" s="39" t="s">
+      <c r="S27" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="T27" s="39" t="s">
+      <c r="T27" s="30" t="s">
         <v>134</v>
       </c>
     </row>
@@ -5016,35 +5018,33 @@
       <c r="B28" s="3">
         <v>7</v>
       </c>
-      <c r="C28" s="81"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="23" t="s">
+      <c r="C28" s="60"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="F28" s="36" t="s">
+      <c r="F28" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="49"/>
-      <c r="M28" s="49"/>
-      <c r="N28" s="49"/>
-      <c r="O28" s="30" t="s">
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="46" t="s">
+        <v>164</v>
+      </c>
+      <c r="O28" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="P28" s="30" t="s">
+      <c r="P28" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="R28" s="46" t="s">
+      <c r="R28" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="S28" s="47" t="s">
+      <c r="S28" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="T28" s="47" t="s">
+      <c r="T28" s="36" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5052,39 +5052,35 @@
       <c r="B29" s="3">
         <v>8</v>
       </c>
-      <c r="C29" s="82" t="s">
+      <c r="C29" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="83"/>
-      <c r="E29" s="23" t="s">
+      <c r="D29" s="62"/>
+      <c r="E29" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="59" t="s">
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="38" t="s">
         <v>146</v>
       </c>
-      <c r="I29" s="61" t="s">
+      <c r="I29" s="39" t="s">
         <v>152</v>
       </c>
-      <c r="J29" s="49"/>
-      <c r="K29" s="49"/>
-      <c r="L29" s="49"/>
-      <c r="M29" s="49"/>
-      <c r="N29" s="49"/>
-      <c r="O29" s="30" t="s">
+      <c r="J29" s="1"/>
+      <c r="O29" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="P29" s="30" t="s">
+      <c r="P29" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="R29" s="46" t="s">
+      <c r="R29" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="S29" s="47" t="s">
+      <c r="S29" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="T29" s="47" t="s">
+      <c r="T29" s="36" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5092,33 +5088,29 @@
       <c r="B30" s="3">
         <v>9</v>
       </c>
-      <c r="C30" s="82"/>
-      <c r="D30" s="83"/>
-      <c r="E30" s="23" t="s">
+      <c r="C30" s="61"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="49"/>
-      <c r="K30" s="49"/>
-      <c r="L30" s="49"/>
-      <c r="M30" s="49"/>
-      <c r="N30" s="49"/>
-      <c r="O30" s="30" t="s">
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="O30" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="P30" s="30" t="s">
+      <c r="P30" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="R30" s="41" t="s">
+      <c r="R30" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="S30" s="40" t="s">
+      <c r="S30" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="T30" s="40" t="s">
+      <c r="T30" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5126,33 +5118,31 @@
       <c r="B31" s="3">
         <v>10</v>
       </c>
-      <c r="C31" s="82"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="23" t="s">
+      <c r="C31" s="61"/>
+      <c r="D31" s="62"/>
+      <c r="E31" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="F31" s="34"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="49"/>
-      <c r="K31" s="49"/>
-      <c r="L31" s="49"/>
-      <c r="M31" s="49"/>
-      <c r="N31" s="49"/>
-      <c r="O31" s="30" t="s">
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="47" t="s">
+        <v>169</v>
+      </c>
+      <c r="O31" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="P31" s="30" t="s">
+      <c r="P31" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="R31" s="41" t="s">
+      <c r="R31" s="32" t="s">
         <v>104</v>
       </c>
-      <c r="S31" s="40" t="s">
+      <c r="S31" s="31" t="s">
         <v>105</v>
       </c>
-      <c r="T31" s="40" t="s">
+      <c r="T31" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5160,33 +5150,29 @@
       <c r="B32" s="3">
         <v>11</v>
       </c>
-      <c r="C32" s="82"/>
-      <c r="D32" s="83"/>
-      <c r="E32" s="23" t="s">
+      <c r="C32" s="61"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="49"/>
-      <c r="L32" s="49"/>
-      <c r="M32" s="49"/>
-      <c r="N32" s="49"/>
-      <c r="O32" s="30" t="s">
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="O32" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="P32" s="30" t="s">
+      <c r="P32" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="R32" s="38" t="s">
+      <c r="R32" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="S32" s="39" t="s">
+      <c r="S32" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="T32" s="39" t="s">
+      <c r="T32" s="30" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5197,92 +5183,82 @@
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
-      <c r="L33" s="49"/>
-      <c r="M33" s="49"/>
-      <c r="N33" s="49"/>
-      <c r="O33" s="30" t="s">
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="47" t="s">
+        <v>168</v>
+      </c>
+      <c r="O33" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="P33" s="30" t="s">
+      <c r="P33" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="R33" s="38" t="s">
+      <c r="R33" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="S33" s="39" t="s">
+      <c r="S33" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="T33" s="39" t="s">
+      <c r="T33" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B34" s="11">
+      <c r="B34" s="10">
         <v>13</v>
       </c>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
-      <c r="L34" s="49"/>
-      <c r="M34" s="49"/>
-      <c r="N34" s="49"/>
-      <c r="O34" s="30" t="s">
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="O34" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="P34" s="30" t="s">
+      <c r="P34" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="R34" s="38" t="s">
+      <c r="R34" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="S34" s="39" t="s">
+      <c r="S34" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="T34" s="39" t="s">
+      <c r="T34" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="B35" s="11">
+      <c r="B35" s="10">
         <v>14</v>
       </c>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="26"/>
-      <c r="I35" s="26"/>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
-      <c r="L35" s="49"/>
-      <c r="M35" s="49"/>
-      <c r="N35" s="49"/>
-      <c r="O35" s="30" t="s">
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="O35" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="P35" s="30" t="s">
+      <c r="P35" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="R35" s="38" t="s">
+      <c r="R35" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="S35" s="39" t="s">
+      <c r="S35" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="T35" s="39" t="s">
+      <c r="T35" s="30" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5293,70 +5269,52 @@
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
-      <c r="L36" s="49"/>
-      <c r="M36" s="49"/>
-      <c r="N36" s="49"/>
-      <c r="O36" s="30" t="s">
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="69"/>
+      <c r="O36" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="P36" s="30" t="s">
+      <c r="P36" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="R36" s="38" t="s">
+      <c r="R36" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="S36" s="39" t="s">
+      <c r="S36" s="30" t="s">
         <v>99</v>
       </c>
-      <c r="T36" s="39" t="s">
+      <c r="T36" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49"/>
-      <c r="M37" s="49"/>
-      <c r="N37" s="49"/>
-      <c r="O37" s="30" t="s">
+      <c r="O37" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="P37" s="30" t="s">
+      <c r="P37" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="R37" s="38" t="s">
+      <c r="R37" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="S37" s="39" t="s">
+      <c r="S37" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="T37" s="39" t="s">
+      <c r="T37" s="30" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="H38" s="49"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="49"/>
-      <c r="K38" s="49"/>
-      <c r="L38" s="49"/>
-      <c r="M38" s="49"/>
-      <c r="N38" s="49"/>
-      <c r="R38" s="38" t="s">
+      <c r="R38" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="S38" s="39" t="s">
+      <c r="S38" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="T38" s="39" t="s">
+      <c r="T38" s="30" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5367,34 +5325,32 @@
       <c r="C39" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="D39" s="68" t="s">
+      <c r="D39" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="E39" s="68"/>
-      <c r="F39" s="30" t="s">
+      <c r="E39" s="49"/>
+      <c r="F39" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G39" s="42" t="s">
+      <c r="G39" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="H39" s="31" t="s">
+      <c r="H39" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I39" s="31" t="s">
+      <c r="I39" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="J39" s="49"/>
-      <c r="K39" s="49"/>
-      <c r="L39" s="49"/>
-      <c r="M39" s="49"/>
-      <c r="N39" s="49"/>
-      <c r="R39" s="38" t="s">
+      <c r="J39" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="R39" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="S39" s="39" t="s">
+      <c r="S39" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="T39" s="39" t="s">
+      <c r="T39" s="30" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5405,26 +5361,24 @@
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="36" t="s">
+      <c r="F40" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="G40" s="45" t="s">
+      <c r="G40" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="H40" s="26"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="49"/>
-      <c r="K40" s="49"/>
-      <c r="L40" s="49"/>
-      <c r="M40" s="49"/>
-      <c r="N40" s="49"/>
-      <c r="R40" s="41" t="s">
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="R40" s="32" t="s">
         <v>118</v>
       </c>
-      <c r="S40" s="40" t="s">
+      <c r="S40" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="T40" s="40" t="s">
+      <c r="T40" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5435,26 +5389,22 @@
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="1"/>
-      <c r="F41" s="36" t="s">
+      <c r="F41" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="G41" s="45" t="s">
+      <c r="G41" s="34" t="s">
         <v>125</v>
       </c>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="49"/>
-      <c r="K41" s="49"/>
-      <c r="L41" s="49"/>
-      <c r="M41" s="49"/>
-      <c r="N41" s="49"/>
-      <c r="R41" s="41" t="s">
+      <c r="H41" s="1"/>
+      <c r="I41" s="1"/>
+      <c r="J41" s="69"/>
+      <c r="R41" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="S41" s="40" t="s">
+      <c r="S41" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="T41" s="40" t="s">
+      <c r="T41" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5467,20 +5417,16 @@
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="49"/>
-      <c r="K42" s="49"/>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
-      <c r="N42" s="49"/>
-      <c r="R42" s="41" t="s">
+      <c r="H42" s="1"/>
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="R42" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="S42" s="40" t="s">
+      <c r="S42" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="T42" s="40" t="s">
+      <c r="T42" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5488,28 +5434,24 @@
       <c r="A43" t="s">
         <v>157</v>
       </c>
-      <c r="B43" s="13">
+      <c r="B43" s="12">
         <v>3</v>
       </c>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="31"/>
-      <c r="I43" s="31"/>
-      <c r="J43" s="49"/>
-      <c r="K43" s="49"/>
-      <c r="L43" s="49"/>
-      <c r="M43" s="49"/>
-      <c r="N43" s="49"/>
-      <c r="R43" s="41" t="s">
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="1"/>
+      <c r="R43" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="S43" s="40" t="s">
+      <c r="S43" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="T43" s="40" t="s">
+      <c r="T43" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5518,30 +5460,26 @@
         <v>4</v>
       </c>
       <c r="C44" s="4"/>
-      <c r="D44" s="87" t="s">
+      <c r="D44" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="E44" s="24" t="s">
+      <c r="E44" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="F44" s="26"/>
-      <c r="G44" s="45" t="s">
+      <c r="F44" s="1"/>
+      <c r="G44" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="H44" s="26"/>
-      <c r="I44" s="26"/>
-      <c r="J44" s="49"/>
-      <c r="K44" s="49"/>
-      <c r="L44" s="49"/>
-      <c r="M44" s="49"/>
-      <c r="N44" s="49"/>
-      <c r="R44" s="41" t="s">
+      <c r="H44" s="1"/>
+      <c r="I44" s="1"/>
+      <c r="J44" s="1"/>
+      <c r="R44" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="S44" s="40" t="s">
+      <c r="S44" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="T44" s="40" t="s">
+      <c r="T44" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5550,28 +5488,24 @@
         <v>5</v>
       </c>
       <c r="C45" s="4"/>
-      <c r="D45" s="87"/>
-      <c r="E45" s="24" t="s">
+      <c r="D45" s="66"/>
+      <c r="E45" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="F45" s="26"/>
-      <c r="G45" s="45" t="s">
+      <c r="F45" s="1"/>
+      <c r="G45" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="H45" s="26"/>
-      <c r="I45" s="26"/>
-      <c r="J45" s="49"/>
-      <c r="K45" s="49"/>
-      <c r="L45" s="49"/>
-      <c r="M45" s="49"/>
-      <c r="N45" s="49"/>
-      <c r="R45" s="41" t="s">
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+      <c r="J45" s="1"/>
+      <c r="R45" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="S45" s="40" t="s">
+      <c r="S45" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="T45" s="40" t="s">
+      <c r="T45" s="31" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5580,210 +5514,167 @@
         <v>6</v>
       </c>
       <c r="C46" s="4"/>
-      <c r="D46" s="87"/>
-      <c r="E46" s="24" t="s">
+      <c r="D46" s="66"/>
+      <c r="E46" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F46" s="26"/>
-      <c r="G46" s="45" t="s">
+      <c r="F46" s="1"/>
+      <c r="G46" s="34" t="s">
         <v>128</v>
       </c>
-      <c r="H46" s="55" t="s">
+      <c r="H46" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="I46" s="26"/>
-      <c r="J46" s="49"/>
-      <c r="K46" s="49"/>
-      <c r="L46" s="49"/>
-      <c r="M46" s="49"/>
-      <c r="N46" s="49"/>
+      <c r="I46" s="1"/>
+      <c r="J46" s="1"/>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B47" s="4">
         <v>7</v>
       </c>
       <c r="C47" s="4"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="24" t="s">
+      <c r="D47" s="66"/>
+      <c r="E47" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="F47" s="26"/>
-      <c r="G47" s="45" t="s">
+      <c r="F47" s="1"/>
+      <c r="G47" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="H47" s="55" t="s">
+      <c r="H47" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="I47" s="26"/>
-      <c r="J47" s="49"/>
-      <c r="K47" s="49"/>
-      <c r="L47" s="49"/>
-      <c r="M47" s="49"/>
-      <c r="N47" s="49"/>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B48" s="4">
         <v>8</v>
       </c>
       <c r="C48" s="4"/>
-      <c r="D48" s="87"/>
-      <c r="E48" s="24" t="s">
+      <c r="D48" s="66"/>
+      <c r="E48" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="F48" s="26"/>
-      <c r="G48" s="45" t="s">
+      <c r="F48" s="1"/>
+      <c r="G48" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="H48" s="26"/>
-      <c r="I48" s="61" t="s">
+      <c r="H48" s="1"/>
+      <c r="I48" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="J48" s="49"/>
-      <c r="K48" s="49"/>
-      <c r="L48" s="49"/>
-      <c r="M48" s="49"/>
-      <c r="N48" s="49"/>
+      <c r="J48" s="1"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B49" s="4">
         <v>9</v>
       </c>
       <c r="C49" s="4"/>
-      <c r="D49" s="87"/>
-      <c r="E49" s="24" t="s">
+      <c r="D49" s="66"/>
+      <c r="E49" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="F49" s="26"/>
-      <c r="G49" s="45" t="s">
+      <c r="F49" s="1"/>
+      <c r="G49" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="H49" s="26"/>
-      <c r="I49" s="61" t="s">
+      <c r="H49" s="1"/>
+      <c r="I49" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="J49" s="49"/>
-      <c r="K49" s="49"/>
-      <c r="L49" s="49"/>
-      <c r="M49" s="49"/>
-      <c r="N49" s="49"/>
+      <c r="J49" s="1"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B50" s="4">
         <v>10</v>
       </c>
       <c r="C50" s="4"/>
-      <c r="D50" s="87"/>
-      <c r="E50" s="24" t="s">
+      <c r="D50" s="66"/>
+      <c r="E50" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
-      <c r="H50" s="26"/>
-      <c r="I50" s="26"/>
-      <c r="J50" s="49"/>
-      <c r="K50" s="49"/>
-      <c r="L50" s="49"/>
-      <c r="M50" s="49"/>
-      <c r="N50" s="49"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>156</v>
       </c>
-      <c r="B51" s="16">
+      <c r="B51" s="15">
         <v>11</v>
       </c>
-      <c r="C51" s="17"/>
-      <c r="D51" s="18"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="18"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="27"/>
-      <c r="J51" s="49"/>
-      <c r="K51" s="49"/>
-      <c r="L51" s="49"/>
-      <c r="M51" s="49"/>
-      <c r="N51" s="49"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="1"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B52" s="4">
         <v>12</v>
       </c>
-      <c r="C52" s="84" t="s">
+      <c r="C52" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="D52" s="15"/>
+      <c r="D52" s="14"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
-      <c r="H52" s="26"/>
-      <c r="I52" s="26"/>
-      <c r="J52" s="49"/>
-      <c r="K52" s="49"/>
-      <c r="L52" s="49"/>
-      <c r="M52" s="49"/>
-      <c r="N52" s="49"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="69"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B53" s="4">
         <v>13</v>
       </c>
-      <c r="C53" s="85"/>
-      <c r="D53" s="15"/>
+      <c r="C53" s="64"/>
+      <c r="D53" s="14"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
-      <c r="H53" s="26"/>
-      <c r="I53" s="26"/>
-      <c r="J53" s="49"/>
-      <c r="K53" s="49"/>
-      <c r="L53" s="49"/>
-      <c r="M53" s="49"/>
-      <c r="N53" s="49"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="19" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B54" s="4">
         <v>14</v>
       </c>
-      <c r="C54" s="85"/>
-      <c r="D54" s="15"/>
+      <c r="C54" s="64"/>
+      <c r="D54" s="14"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
-      <c r="H54" s="26"/>
-      <c r="I54" s="26"/>
-      <c r="J54" s="49"/>
-      <c r="K54" s="49"/>
-      <c r="L54" s="49"/>
-      <c r="M54" s="49"/>
-      <c r="N54" s="49"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="19" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B55" s="4">
         <v>15</v>
       </c>
-      <c r="C55" s="86"/>
-      <c r="D55" s="15"/>
+      <c r="C55" s="65"/>
+      <c r="D55" s="14"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="26"/>
-      <c r="J55" s="49"/>
-      <c r="K55" s="49"/>
-      <c r="L55" s="49"/>
-      <c r="M55" s="49"/>
-      <c r="N55" s="49"/>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="H56" s="49"/>
-      <c r="I56" s="49"/>
-      <c r="J56" s="49"/>
-      <c r="K56" s="49"/>
-      <c r="L56" s="49"/>
-      <c r="M56" s="49"/>
-      <c r="N56" s="49"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="19" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B58" s="4" t="s">
@@ -5795,196 +5686,178 @@
       <c r="D58" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E58" s="74" t="s">
+      <c r="E58" s="55" t="s">
         <v>70</v>
       </c>
-      <c r="F58" s="75"/>
-      <c r="G58" s="68" t="s">
+      <c r="F58" s="56"/>
+      <c r="G58" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="H58" s="68"/>
-      <c r="I58" s="31" t="s">
+      <c r="H58" s="49"/>
+      <c r="I58" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="J58" s="31" t="s">
+      <c r="J58" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="K58" s="31" t="s">
+      <c r="K58" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="L58" s="53"/>
-      <c r="M58" s="53"/>
-      <c r="N58" s="53"/>
+      <c r="L58" s="18"/>
+      <c r="M58" s="18"/>
+      <c r="N58" s="18"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B59" s="4">
         <v>0</v>
       </c>
-      <c r="C59" s="79" t="s">
+      <c r="C59" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="D59" s="80" t="s">
+      <c r="D59" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="14"/>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
-      <c r="I59" s="36" t="s">
+      <c r="I59" s="27" t="s">
         <v>80</v>
       </c>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
-      <c r="L59" s="60"/>
-      <c r="M59" s="60"/>
-      <c r="N59" s="60"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B60" s="4">
         <v>1</v>
       </c>
-      <c r="C60" s="79"/>
-      <c r="D60" s="80"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
+      <c r="C60" s="58"/>
+      <c r="D60" s="59"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
-      <c r="I60" s="36" t="s">
+      <c r="I60" s="27" t="s">
         <v>81</v>
       </c>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
-      <c r="L60" s="60"/>
-      <c r="M60" s="60"/>
-      <c r="N60" s="60"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B61" s="4">
         <v>2</v>
       </c>
-      <c r="C61" s="79"/>
-      <c r="D61" s="80"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
+      <c r="C61" s="58"/>
+      <c r="D61" s="59"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="14"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
-      <c r="I61" s="36" t="s">
+      <c r="I61" s="27" t="s">
         <v>82</v>
       </c>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
-      <c r="L61" s="60"/>
-      <c r="M61" s="60"/>
-      <c r="N61" s="60"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B62" s="4">
         <v>3</v>
       </c>
-      <c r="C62" s="79"/>
-      <c r="D62" s="80"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="15"/>
+      <c r="C62" s="58"/>
+      <c r="D62" s="59"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="14"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
-      <c r="I62" s="36" t="s">
+      <c r="I62" s="27" t="s">
         <v>83</v>
       </c>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
-      <c r="L62" s="60"/>
-      <c r="M62" s="60"/>
-      <c r="N62" s="60"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B63" s="4">
         <v>4</v>
       </c>
-      <c r="C63" s="79"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
+      <c r="C63" s="58"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14"/>
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
-      <c r="I63" s="36" t="s">
+      <c r="I63" s="27" t="s">
         <v>84</v>
       </c>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
-      <c r="L63" s="60"/>
-      <c r="M63" s="60"/>
-      <c r="N63" s="60"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B64" s="4">
         <v>5</v>
       </c>
-      <c r="C64" s="79"/>
-      <c r="D64" s="15"/>
-      <c r="E64" s="89" t="s">
+      <c r="C64" s="58"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="F64" s="21" t="s">
+      <c r="F64" s="19" t="s">
         <v>27</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
-      <c r="I64" s="36" t="s">
+      <c r="I64" s="27" t="s">
         <v>85</v>
       </c>
       <c r="J64" s="1"/>
-      <c r="K64" s="26"/>
-      <c r="L64" s="50"/>
-      <c r="M64" s="50"/>
-      <c r="N64" s="50"/>
+      <c r="K64" s="1"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B65" s="4">
         <v>6</v>
       </c>
-      <c r="C65" s="79"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="90"/>
-      <c r="F65" s="21" t="s">
+      <c r="C65" s="58"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="68"/>
+      <c r="F65" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="G65" s="71" t="s">
+      <c r="G65" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="H65" s="22" t="s">
+      <c r="H65" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I65" s="1"/>
-      <c r="J65" s="55" t="s">
+      <c r="J65" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="K65" s="54"/>
-      <c r="L65" s="51"/>
-      <c r="M65" s="51"/>
-      <c r="N65" s="51"/>
+      <c r="K65" s="3"/>
+      <c r="L65" s="5"/>
+      <c r="M65" s="5"/>
+      <c r="N65" s="5"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B66" s="4">
         <v>7</v>
       </c>
-      <c r="C66" s="79"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="90"/>
-      <c r="F66" s="21" t="s">
+      <c r="C66" s="58"/>
+      <c r="D66" s="14"/>
+      <c r="E66" s="68"/>
+      <c r="F66" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G66" s="72"/>
-      <c r="H66" s="22" t="s">
+      <c r="G66" s="53"/>
+      <c r="H66" s="20" t="s">
         <v>20</v>
       </c>
       <c r="I66" s="1"/>
-      <c r="J66" s="55" t="s">
+      <c r="J66" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="K66" s="54"/>
-      <c r="L66" s="51"/>
-      <c r="M66" s="51"/>
-      <c r="N66" s="51"/>
+      <c r="K66" s="3"/>
+      <c r="L66" s="5"/>
+      <c r="M66" s="5"/>
+      <c r="N66" s="5"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B67" s="4">
@@ -5992,22 +5865,19 @@
       </c>
       <c r="C67" s="4"/>
       <c r="D67" s="4"/>
-      <c r="E67" s="90"/>
-      <c r="F67" s="21" t="s">
+      <c r="E67" s="68"/>
+      <c r="F67" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="G67" s="72"/>
-      <c r="H67" s="22" t="s">
+      <c r="G67" s="53"/>
+      <c r="H67" s="20" t="s">
         <v>21</v>
       </c>
       <c r="I67" s="1"/>
-      <c r="J67" s="59" t="s">
+      <c r="J67" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="K67" s="26"/>
-      <c r="L67" s="50"/>
-      <c r="M67" s="50"/>
-      <c r="N67" s="50"/>
+      <c r="K67" s="1"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B68" s="4">
@@ -6015,22 +5885,19 @@
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
-      <c r="E68" s="90"/>
-      <c r="F68" s="21" t="s">
+      <c r="E68" s="68"/>
+      <c r="F68" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G68" s="72"/>
-      <c r="H68" s="22" t="s">
+      <c r="G68" s="53"/>
+      <c r="H68" s="20" t="s">
         <v>25</v>
       </c>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
-      <c r="K68" s="61" t="s">
+      <c r="K68" s="39" t="s">
         <v>150</v>
       </c>
-      <c r="L68" s="50"/>
-      <c r="M68" s="50"/>
-      <c r="N68" s="50"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B69" s="4">
@@ -6038,20 +5905,17 @@
       </c>
       <c r="C69" s="4"/>
       <c r="D69" s="4"/>
-      <c r="E69" s="90"/>
-      <c r="F69" s="21" t="s">
+      <c r="E69" s="68"/>
+      <c r="F69" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="G69" s="72"/>
-      <c r="H69" s="22" t="s">
+      <c r="G69" s="53"/>
+      <c r="H69" s="20" t="s">
         <v>24</v>
       </c>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
-      <c r="L69" s="60"/>
-      <c r="M69" s="60"/>
-      <c r="N69" s="60"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B70" s="4">
@@ -6059,20 +5923,17 @@
       </c>
       <c r="C70" s="4"/>
       <c r="D70" s="4"/>
-      <c r="E70" s="90"/>
-      <c r="F70" s="21" t="s">
+      <c r="E70" s="68"/>
+      <c r="F70" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="G70" s="72"/>
-      <c r="H70" s="22" t="s">
+      <c r="G70" s="53"/>
+      <c r="H70" s="20" t="s">
         <v>23</v>
       </c>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
-      <c r="L70" s="60"/>
-      <c r="M70" s="60"/>
-      <c r="N70" s="60"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B71" s="4">
@@ -6080,74 +5941,62 @@
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="4"/>
-      <c r="E71" s="90"/>
-      <c r="F71" s="21" t="s">
+      <c r="E71" s="68"/>
+      <c r="F71" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="G71" s="73"/>
-      <c r="H71" s="22" t="s">
+      <c r="G71" s="54"/>
+      <c r="H71" s="20" t="s">
         <v>22</v>
       </c>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
-      <c r="L71" s="60"/>
-      <c r="M71" s="60"/>
-      <c r="N71" s="60"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B72" s="29">
+      <c r="B72" s="24">
         <v>13</v>
       </c>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="27"/>
-      <c r="H72" s="26"/>
+      <c r="E72" s="23"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="14"/>
+      <c r="H72" s="1"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
-      <c r="L72" s="60"/>
-      <c r="M72" s="60"/>
-      <c r="N72" s="60"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B73" s="13">
+      <c r="B73" s="12">
         <v>14</v>
       </c>
-      <c r="C73" s="13"/>
-      <c r="D73" s="13"/>
-      <c r="E73" s="13"/>
-      <c r="F73" s="13"/>
-      <c r="G73" s="12"/>
-      <c r="H73" s="12"/>
-      <c r="I73" s="12"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
       <c r="J73" s="1"/>
       <c r="K73" s="1"/>
-      <c r="L73" s="60"/>
-      <c r="M73" s="60"/>
-      <c r="N73" s="60"/>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B74" s="13">
+      <c r="B74" s="12">
         <v>15</v>
       </c>
-      <c r="C74" s="13"/>
-      <c r="D74" s="13"/>
-      <c r="E74" s="13"/>
-      <c r="F74" s="13"/>
-      <c r="G74" s="12"/>
-      <c r="H74" s="12"/>
-      <c r="I74" s="12"/>
+      <c r="C74" s="12"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="12"/>
+      <c r="F74" s="12"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
-      <c r="L74" s="60"/>
-      <c r="M74" s="60"/>
-      <c r="N74" s="60"/>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B77" s="4" t="s">
@@ -6159,8 +6008,26 @@
         <v>2</v>
       </c>
     </row>
+    <row r="86" spans="20:25" x14ac:dyDescent="0.3">
+      <c r="T86" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="U86" s="48"/>
+      <c r="V86" s="48"/>
+      <c r="W86" s="48"/>
+      <c r="X86" s="48"/>
+      <c r="Y86" s="48"/>
+    </row>
+    <row r="87" spans="20:25" x14ac:dyDescent="0.3">
+      <c r="T87" s="48"/>
+      <c r="U87" s="48"/>
+      <c r="V87" s="48"/>
+      <c r="W87" s="48"/>
+      <c r="X87" s="48"/>
+      <c r="Y87" s="48"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="C59:C66"/>
     <mergeCell ref="D59:D62"/>
@@ -6173,6 +6040,7 @@
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="E58:F58"/>
     <mergeCell ref="E64:E71"/>
+    <mergeCell ref="T86:Y87"/>
     <mergeCell ref="R14:S14"/>
     <mergeCell ref="O13:S13"/>
     <mergeCell ref="R22:T22"/>

</xml_diff>